<commit_message>
Generate Self Employed packages from app/data and app/templates
Triggered by: 153ec27ed63cc8a45dbe5e2a9efc7bd6d6d1ed85
</commit_message>
<xml_diff>
--- a/examples/ltd-latest/Financialaccounts.xlsx
+++ b/examples/ltd-latest/Financialaccounts.xlsx
@@ -43133,7 +43133,7 @@
       <c r="B57" s="129"/>
       <c r="C57" s="130" t="n">
         <f aca="true">TODAY()</f>
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="D57" s="130"/>
     </row>
@@ -43966,7 +43966,7 @@
       </c>
       <c r="D74" s="152" t="n">
         <f aca="true">TODAY()</f>
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="E74" s="152"/>
       <c r="F74" s="152"/>
@@ -44508,7 +44508,7 @@
       </c>
       <c r="G119" s="159" t="n">
         <f aca="true">TODAY()</f>
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="H119" s="159"/>
     </row>

</xml_diff>